<commit_message>
Add Lightbox feature with labels to About Us images
</commit_message>
<xml_diff>
--- a/FFE_schedule_professional.xlsx
+++ b/FFE_schedule_professional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\PROJECTS\UMA BALI CZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7919D1F8-97ED-4DE1-9D7B-D8BB594707B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED797C6-F31F-4F68-89A2-D3FE90E7A789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1739,6 +1739,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{E7E08E70-4AD4-4DC7-99EA-547BA0961B49}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;b39ab285-c221-42d1-99aa-06df5ba9faba&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O90"/>

</xml_diff>